<commit_message>
updating csvs from corrected databases
</commit_message>
<xml_diff>
--- a/Data for R/FLaSH/FLaSH EDI Qry_Empties with Enviro.xlsx
+++ b/Data for R/FLaSH/FLaSH EDI Qry_Empties with Enviro.xlsx
@@ -888,7 +888,7 @@
       <c r="N2" s="9">
         <v>5.91239763594603</v>
       </c>
-      <c r="O2" s="9">
+      <c r="O2" s="10">
         <v>27</v>
       </c>
       <c r="P2" s="9">
@@ -976,7 +976,7 @@
       <c r="N3" s="9">
         <v>7.61106010654548</v>
       </c>
-      <c r="O3" s="9">
+      <c r="O3" s="10">
         <v>46</v>
       </c>
       <c r="P3" s="9">
@@ -1067,7 +1067,7 @@
       <c r="N4" s="9">
         <v>8.93932597090552</v>
       </c>
-      <c r="O4" s="9">
+      <c r="O4" s="10">
         <v>66</v>
       </c>
       <c r="P4" s="9">
@@ -1158,7 +1158,7 @@
       <c r="N5" s="9">
         <v>0.233956419909353</v>
       </c>
-      <c r="O5" s="9">
+      <c r="O5" s="10">
         <v>17</v>
       </c>
       <c r="P5" s="9">
@@ -1249,7 +1249,7 @@
       <c r="N6" s="9">
         <v>0.29</v>
       </c>
-      <c r="O6" s="9">
+      <c r="O6" s="10">
         <v>43</v>
       </c>
       <c r="P6" s="9">
@@ -1340,7 +1340,7 @@
       <c r="N7" s="9">
         <v>0.56</v>
       </c>
-      <c r="O7" s="9">
+      <c r="O7" s="10">
         <v>20</v>
       </c>
       <c r="P7" s="9">
@@ -1431,7 +1431,7 @@
       <c r="N8" s="9">
         <v>0.56</v>
       </c>
-      <c r="O8" s="9">
+      <c r="O8" s="10">
         <v>20</v>
       </c>
       <c r="P8" s="9">
@@ -1522,7 +1522,7 @@
       <c r="N9" s="9">
         <v>0.07</v>
       </c>
-      <c r="O9" s="9">
+      <c r="O9" s="10">
         <v>81</v>
       </c>
       <c r="P9" s="9">
@@ -1613,7 +1613,7 @@
       <c r="N10" s="9">
         <v>0.14</v>
       </c>
-      <c r="O10" s="9">
+      <c r="O10" s="10">
         <v>34</v>
       </c>
       <c r="P10" s="9">
@@ -1704,7 +1704,7 @@
       <c r="N11" s="9">
         <v>0.08</v>
       </c>
-      <c r="O11" s="9">
+      <c r="O11" s="10">
         <v>32</v>
       </c>
       <c r="P11" s="9">
@@ -1795,7 +1795,7 @@
       <c r="N12" s="9">
         <v>0.116266663217221</v>
       </c>
-      <c r="O12" s="9">
+      <c r="O12" s="10">
         <v>72</v>
       </c>
       <c r="P12" s="9">
@@ -1889,7 +1889,7 @@
       <c r="N13" s="9">
         <v>4.30947075014608</v>
       </c>
-      <c r="O13" s="9">
+      <c r="O13" s="10">
         <v>40</v>
       </c>
       <c r="Q13" s="9">
@@ -1980,7 +1980,7 @@
       <c r="N14" s="9">
         <v>4.30947075014608</v>
       </c>
-      <c r="O14" s="9">
+      <c r="O14" s="10">
         <v>40</v>
       </c>
       <c r="Q14" s="9">
@@ -2071,7 +2071,7 @@
       <c r="N15" s="9">
         <v>6.57823246724982</v>
       </c>
-      <c r="O15" s="9">
+      <c r="O15" s="10">
         <v>22</v>
       </c>
       <c r="Q15" s="9">
@@ -2162,7 +2162,7 @@
       <c r="N16" s="9">
         <v>4.22113673098982</v>
       </c>
-      <c r="O16" s="9">
+      <c r="O16" s="10">
         <v>30</v>
       </c>
       <c r="Q16" s="9">
@@ -2253,7 +2253,7 @@
       <c r="N17" s="9">
         <v>0.714149189200495</v>
       </c>
-      <c r="O17" s="9">
+      <c r="O17" s="10">
         <v>27</v>
       </c>
       <c r="Q17" s="9">
@@ -2344,7 +2344,7 @@
       <c r="N18" s="9">
         <v>0.181581224941503</v>
       </c>
-      <c r="O18" s="9">
+      <c r="O18" s="10">
         <v>28</v>
       </c>
       <c r="Q18" s="9">
@@ -2435,7 +2435,7 @@
       <c r="N19" s="9">
         <v>0.181581224941503</v>
       </c>
-      <c r="O19" s="9">
+      <c r="O19" s="10">
         <v>28</v>
       </c>
       <c r="Q19" s="9">
@@ -2526,7 +2526,7 @@
       <c r="N20" s="9">
         <v>0.733996912617268</v>
       </c>
-      <c r="O20" s="9">
+      <c r="O20" s="10">
         <v>44</v>
       </c>
       <c r="P20" s="9">
@@ -2620,7 +2620,7 @@
       <c r="N21" s="9">
         <v>0.628411617</v>
       </c>
-      <c r="O21" s="9">
+      <c r="O21" s="10">
         <v>20</v>
       </c>
       <c r="P21" s="9">
@@ -2714,7 +2714,7 @@
       <c r="N22" s="9">
         <v>2.243137285</v>
       </c>
-      <c r="O22" s="9">
+      <c r="O22" s="10">
         <v>27</v>
       </c>
       <c r="P22" s="9">
@@ -2808,7 +2808,7 @@
       <c r="N23" s="9">
         <v>0.751786255</v>
       </c>
-      <c r="O23" s="9">
+      <c r="O23" s="10">
         <v>17</v>
       </c>
       <c r="P23" s="9">
@@ -2902,7 +2902,7 @@
       <c r="N24" s="9">
         <v>0.733996912617268</v>
       </c>
-      <c r="O24" s="9">
+      <c r="O24" s="10">
         <v>44</v>
       </c>
       <c r="P24" s="9">
@@ -2996,7 +2996,7 @@
       <c r="N25" s="9">
         <v>7.07014200626035E-02</v>
       </c>
-      <c r="O25" s="9">
+      <c r="O25" s="10">
         <v>43</v>
       </c>
       <c r="Q25" s="9">
@@ -3087,7 +3087,7 @@
       <c r="N26" s="9">
         <v>6.54016567157918</v>
       </c>
-      <c r="O26" s="9">
+      <c r="O26" s="10">
         <v>19</v>
       </c>
       <c r="Q26" s="9">
@@ -3184,7 +3184,7 @@
       <c r="N27" s="9">
         <v>6.54016567157918</v>
       </c>
-      <c r="O27" s="9">
+      <c r="O27" s="10">
         <v>19</v>
       </c>
       <c r="Q27" s="9">
@@ -3275,7 +3275,7 @@
       <c r="N28" s="9">
         <v>6.54016567157918</v>
       </c>
-      <c r="O28" s="9">
+      <c r="O28" s="10">
         <v>19</v>
       </c>
       <c r="Q28" s="9">
@@ -3366,7 +3366,7 @@
       <c r="N29" s="9">
         <v>9.16612204170404</v>
       </c>
-      <c r="O29" s="9">
+      <c r="O29" s="10">
         <v>18</v>
       </c>
       <c r="Q29" s="9">
@@ -3457,7 +3457,7 @@
       <c r="N30" s="9">
         <v>9.16612204170404</v>
       </c>
-      <c r="O30" s="9">
+      <c r="O30" s="10">
         <v>18</v>
       </c>
       <c r="Q30" s="9">
@@ -3548,7 +3548,7 @@
       <c r="N31" s="9">
         <v>9.16612204170404</v>
       </c>
-      <c r="O31" s="9">
+      <c r="O31" s="10">
         <v>18</v>
       </c>
       <c r="Q31" s="9">
@@ -3639,7 +3639,7 @@
       <c r="N32" s="9">
         <v>9.16612204170404</v>
       </c>
-      <c r="O32" s="9">
+      <c r="O32" s="10">
         <v>18</v>
       </c>
       <c r="Q32" s="9">
@@ -3730,7 +3730,7 @@
       <c r="N33" s="9">
         <v>10.4626731003908</v>
       </c>
-      <c r="O33" s="9">
+      <c r="O33" s="10">
         <v>10</v>
       </c>
       <c r="Q33" s="9">
@@ -3821,7 +3821,7 @@
       <c r="N34" s="9">
         <v>10.4626731003908</v>
       </c>
-      <c r="O34" s="9">
+      <c r="O34" s="10">
         <v>10</v>
       </c>
       <c r="Q34" s="9">
@@ -3912,7 +3912,7 @@
       <c r="N35" s="9">
         <v>0.146101890125461</v>
       </c>
-      <c r="O35" s="9">
+      <c r="O35" s="10">
         <v>63</v>
       </c>
       <c r="Q35" s="9">
@@ -4003,7 +4003,7 @@
       <c r="N36" s="9">
         <v>0.339467723207604</v>
       </c>
-      <c r="O36" s="9">
+      <c r="O36" s="10">
         <v>33</v>
       </c>
       <c r="P36" s="9">
@@ -4097,7 +4097,7 @@
       <c r="N37" s="9">
         <v>0.958821325062239</v>
       </c>
-      <c r="O37" s="9">
+      <c r="O37" s="10">
         <v>36</v>
       </c>
       <c r="P37" s="9">
@@ -4191,7 +4191,7 @@
       <c r="N38" s="9">
         <v>3.55899409093209</v>
       </c>
-      <c r="O38" s="9">
+      <c r="O38" s="10">
         <v>30</v>
       </c>
       <c r="P38" s="9">
@@ -4285,7 +4285,7 @@
       <c r="N39" s="9">
         <v>1.17275584161783</v>
       </c>
-      <c r="O39" s="9">
+      <c r="O39" s="10">
         <v>49.0000009536743</v>
       </c>
       <c r="P39" s="9">
@@ -4379,7 +4379,7 @@
       <c r="N40" s="9">
         <v>8.96570505211038E-02</v>
       </c>
-      <c r="O40" s="9">
+      <c r="O40" s="10">
         <v>38</v>
       </c>
       <c r="P40" s="9">
@@ -4473,7 +4473,7 @@
       <c r="N41" s="9">
         <v>0.754928529738625</v>
       </c>
-      <c r="O41" s="9">
+      <c r="O41" s="10">
         <v>48</v>
       </c>
       <c r="P41" s="9">
@@ -4567,7 +4567,7 @@
       <c r="N42" s="9">
         <v>1.70968314202846</v>
       </c>
-      <c r="O42" s="9">
+      <c r="O42" s="10">
         <v>41</v>
       </c>
       <c r="P42" s="9">
@@ -4661,7 +4661,7 @@
       <c r="N43" s="9">
         <v>1.70968314202846</v>
       </c>
-      <c r="O43" s="9">
+      <c r="O43" s="10">
         <v>41</v>
       </c>
       <c r="P43" s="9">
@@ -4755,7 +4755,7 @@
       <c r="N44" s="9">
         <v>2.2160294728127</v>
       </c>
-      <c r="O44" s="9">
+      <c r="O44" s="10">
         <v>36</v>
       </c>
       <c r="P44" s="9">
@@ -4849,7 +4849,7 @@
       <c r="N45" s="9">
         <v>2.2160294728127</v>
       </c>
-      <c r="O45" s="9">
+      <c r="O45" s="10">
         <v>36</v>
       </c>
       <c r="P45" s="9">
@@ -4943,7 +4943,7 @@
       <c r="N46" s="9">
         <v>2.2160294728127</v>
       </c>
-      <c r="O46" s="9">
+      <c r="O46" s="10">
         <v>36</v>
       </c>
       <c r="P46" s="9">
@@ -5037,7 +5037,7 @@
       <c r="N47" s="9">
         <v>1.75849732530641</v>
       </c>
-      <c r="O47" s="9">
+      <c r="O47" s="10">
         <v>37</v>
       </c>
       <c r="P47" s="9">
@@ -5131,7 +5131,7 @@
       <c r="N48" s="9">
         <v>1.75849732530641</v>
       </c>
-      <c r="O48" s="9">
+      <c r="O48" s="10">
         <v>37</v>
       </c>
       <c r="P48" s="9">
@@ -5225,7 +5225,7 @@
       <c r="N49" s="9">
         <v>0.189213103613724</v>
       </c>
-      <c r="O49" s="9">
+      <c r="O49" s="10">
         <v>39</v>
       </c>
       <c r="P49" s="9">
@@ -5319,7 +5319,7 @@
       <c r="N50" s="9">
         <v>0.189213103613724</v>
       </c>
-      <c r="O50" s="9">
+      <c r="O50" s="10">
         <v>39</v>
       </c>
       <c r="P50" s="9">
@@ -5413,7 +5413,7 @@
       <c r="N51" s="9">
         <v>10.9414851434528</v>
       </c>
-      <c r="O51" s="9">
+      <c r="O51" s="10">
         <v>21</v>
       </c>
       <c r="P51" s="9">
@@ -5507,7 +5507,7 @@
       <c r="N52" s="9">
         <v>10.9414851434528</v>
       </c>
-      <c r="O52" s="9">
+      <c r="O52" s="10">
         <v>21</v>
       </c>
       <c r="P52" s="9">
@@ -5601,7 +5601,7 @@
       <c r="N53" s="9">
         <v>10.9414851434528</v>
       </c>
-      <c r="O53" s="9">
+      <c r="O53" s="10">
         <v>21</v>
       </c>
       <c r="P53" s="9">
@@ -5695,7 +5695,7 @@
       <c r="N54" s="9">
         <v>10.9414851434528</v>
       </c>
-      <c r="O54" s="9">
+      <c r="O54" s="10">
         <v>21</v>
       </c>
       <c r="P54" s="9">
@@ -5789,7 +5789,7 @@
       <c r="N55" s="9">
         <v>0.07</v>
       </c>
-      <c r="O55" s="9">
+      <c r="O55" s="10">
         <v>12</v>
       </c>
       <c r="P55" s="9">
@@ -5841,7 +5841,7 @@
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>FMWTCC</t>
+          <t>MWTCC</t>
         </is>
       </c>
       <c r="D56" s="6">
@@ -5880,7 +5880,7 @@
       <c r="N56" s="9">
         <v>0.6</v>
       </c>
-      <c r="O56" s="9">
+      <c r="O56" s="10">
         <v>0.6</v>
       </c>
       <c r="P56" s="9">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>FMWTCC</t>
+          <t>MWTCC</t>
         </is>
       </c>
       <c r="D57" s="6">
@@ -5971,7 +5971,7 @@
       <c r="N57" s="9">
         <v>0.6</v>
       </c>
-      <c r="O57" s="9">
+      <c r="O57" s="10">
         <v>0.6</v>
       </c>
       <c r="P57" s="9">
@@ -6062,7 +6062,7 @@
       <c r="N58" s="9">
         <v>2.32</v>
       </c>
-      <c r="O58" s="9">
+      <c r="O58" s="10">
         <v>0.59</v>
       </c>
       <c r="P58" s="9">
@@ -6156,7 +6156,7 @@
       <c r="N59" s="9">
         <v>0.58</v>
       </c>
-      <c r="O59" s="9">
+      <c r="O59" s="10">
         <v>0.66</v>
       </c>
       <c r="P59" s="9">
@@ -6250,7 +6250,7 @@
       <c r="N60" s="9">
         <v>1.03</v>
       </c>
-      <c r="O60" s="9">
+      <c r="O60" s="10">
         <v>0.54</v>
       </c>
       <c r="P60" s="9">
@@ -6344,7 +6344,7 @@
       <c r="N61" s="9">
         <v>1.63</v>
       </c>
-      <c r="O61" s="9">
+      <c r="O61" s="10">
         <v>0.57</v>
       </c>
       <c r="P61" s="9">
@@ -6435,7 +6435,7 @@
       <c r="N62" s="9">
         <v>2.32</v>
       </c>
-      <c r="O62" s="9">
+      <c r="O62" s="10">
         <v>0.59</v>
       </c>
       <c r="P62" s="9">
@@ -6529,7 +6529,7 @@
       <c r="N63" s="9">
         <v>0.58</v>
       </c>
-      <c r="O63" s="9">
+      <c r="O63" s="10">
         <v>0.66</v>
       </c>
       <c r="P63" s="9">
@@ -6623,7 +6623,7 @@
       <c r="N64" s="9">
         <v>1.03</v>
       </c>
-      <c r="O64" s="9">
+      <c r="O64" s="10">
         <v>0.54</v>
       </c>
       <c r="P64" s="9">
@@ -6717,7 +6717,7 @@
       <c r="N65" s="9">
         <v>1.63</v>
       </c>
-      <c r="O65" s="9">
+      <c r="O65" s="10">
         <v>0.57</v>
       </c>
       <c r="P65" s="9">
@@ -6811,7 +6811,7 @@
       <c r="N66" s="9">
         <v>0.25</v>
       </c>
-      <c r="O66" s="9">
+      <c r="O66" s="10">
         <v>0.45</v>
       </c>
       <c r="P66" s="9">
@@ -6905,7 +6905,7 @@
       <c r="N67" s="9">
         <v>0.25</v>
       </c>
-      <c r="O67" s="9">
+      <c r="O67" s="10">
         <v>0.45</v>
       </c>
       <c r="P67" s="9">
@@ -6999,7 +6999,7 @@
       <c r="N68" s="9">
         <v>1.42</v>
       </c>
-      <c r="O68" s="9">
+      <c r="O68" s="10">
         <v>0.62</v>
       </c>
       <c r="P68" s="9">
@@ -7093,7 +7093,7 @@
       <c r="N69" s="9">
         <v>1.61</v>
       </c>
-      <c r="O69" s="9">
+      <c r="O69" s="10">
         <v>0.47</v>
       </c>
       <c r="P69" s="9">
@@ -7187,7 +7187,7 @@
       <c r="N70" s="9">
         <v>1.34</v>
       </c>
-      <c r="O70" s="9">
+      <c r="O70" s="10">
         <v>0.48</v>
       </c>
       <c r="P70" s="9">
@@ -7281,7 +7281,7 @@
       <c r="N71" s="9">
         <v>0.98</v>
       </c>
-      <c r="O71" s="9">
+      <c r="O71" s="10">
         <v>0.42</v>
       </c>
       <c r="P71" s="9">
@@ -7375,7 +7375,7 @@
       <c r="N72" s="9">
         <v>0.74</v>
       </c>
-      <c r="O72" s="9">
+      <c r="O72" s="10">
         <v>0.53</v>
       </c>
       <c r="P72" s="9">
@@ -7469,7 +7469,7 @@
       <c r="N73" s="9">
         <v>6.17</v>
       </c>
-      <c r="O73" s="9">
+      <c r="O73" s="10">
         <v>16</v>
       </c>
       <c r="P73" s="9">
@@ -7563,7 +7563,7 @@
       <c r="N74" s="9">
         <v>0.747074510833752</v>
       </c>
-      <c r="O74" s="9">
+      <c r="O74" s="10">
         <v>37.0000004768372</v>
       </c>
       <c r="P74" s="9">
@@ -7657,7 +7657,7 @@
       <c r="N75" s="9">
         <v>0.1</v>
       </c>
-      <c r="O75" s="9">
+      <c r="O75" s="10">
         <v>56</v>
       </c>
       <c r="P75" s="9">
@@ -7751,7 +7751,7 @@
       <c r="N76" s="9">
         <v>0.1</v>
       </c>
-      <c r="O76" s="9">
+      <c r="O76" s="10">
         <v>56</v>
       </c>
       <c r="P76" s="9">
@@ -7845,7 +7845,7 @@
       <c r="N77" s="9">
         <v>0.1</v>
       </c>
-      <c r="O77" s="9">
+      <c r="O77" s="10">
         <v>56</v>
       </c>
       <c r="P77" s="9">

</xml_diff>

<commit_message>
more database updates plus coding for error codes for future
</commit_message>
<xml_diff>
--- a/Data for R/FLaSH/FLaSH EDI Qry_Empties with Enviro.xlsx
+++ b/Data for R/FLaSH/FLaSH EDI Qry_Empties with Enviro.xlsx
@@ -672,7 +672,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z77"/>
+  <dimension ref="A1:AB77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col customWidth="true" min="1" max="1" width="13.62109375"/>
@@ -701,6 +701,8 @@
     <col customWidth="true" min="24" max="24" width="14.0625"/>
     <col customWidth="true" min="25" max="25" width="13.76953125"/>
     <col customWidth="true" min="26" max="26" width="14.0625"/>
+    <col customWidth="true" min="27" max="27" width="10.10546875"/>
+    <col customWidth="true" min="28" max="28" width="10.984375"/>
   </cols>
   <sheetData>
     <row outlineLevel="0" r="1">
@@ -834,6 +836,16 @@
           <t>CulturedOrigin</t>
         </is>
       </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>DietStudy</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>PreyItemsID'd</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="2">
       <c r="A2" s="4">
@@ -922,6 +934,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA2" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="3">
       <c r="A3" s="4">
@@ -1013,6 +1033,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA3" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="4">
       <c r="A4" s="4">
@@ -1104,6 +1132,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA4" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="5">
       <c r="A5" s="4">
@@ -1195,6 +1231,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA5" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="6">
       <c r="A6" s="4">
@@ -1286,6 +1330,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA6" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="7">
       <c r="A7" s="4">
@@ -1377,6 +1429,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA7" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="8">
       <c r="A8" s="4">
@@ -1468,6 +1528,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA8" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="9">
       <c r="A9" s="4">
@@ -1559,6 +1627,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA9" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="10">
       <c r="A10" s="4">
@@ -1650,6 +1726,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA10" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB10" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="11">
       <c r="A11" s="4">
@@ -1741,6 +1825,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA11" s="12">
+        <v>2</v>
+      </c>
+      <c r="AB11" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="12">
       <c r="A12" s="4">
@@ -1835,6 +1927,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA12" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="13">
       <c r="A13" s="4">
@@ -1926,6 +2026,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA13" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB13" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="14">
       <c r="A14" s="4">
@@ -2017,6 +2125,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA14" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="15">
       <c r="A15" s="4">
@@ -2108,6 +2224,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA15" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB15" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="16">
       <c r="A16" s="4">
@@ -2199,6 +2323,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA16" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB16" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="17">
       <c r="A17" s="4">
@@ -2290,6 +2422,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA17" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB17" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="18">
       <c r="A18" s="4">
@@ -2381,6 +2521,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA18" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB18" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="19">
       <c r="A19" s="4">
@@ -2472,6 +2620,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA19" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB19" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="20">
       <c r="A20" s="4">
@@ -2566,6 +2722,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA20" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB20" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="21">
       <c r="A21" s="4">
@@ -2660,6 +2824,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA21" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB21" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="22">
       <c r="A22" s="4">
@@ -2754,6 +2926,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA22" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB22" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="23">
       <c r="A23" s="4">
@@ -2848,6 +3028,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA23" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB23" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="24">
       <c r="A24" s="4">
@@ -2942,6 +3130,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA24" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB24" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="25">
       <c r="A25" s="4">
@@ -3033,6 +3229,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA25" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB25" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="26">
       <c r="A26" s="4">
@@ -3130,6 +3334,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA26" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB26" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="27">
       <c r="A27" s="4">
@@ -3221,6 +3433,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA27" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="28">
       <c r="A28" s="4">
@@ -3312,6 +3532,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA28" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB28" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="29">
       <c r="A29" s="4">
@@ -3403,6 +3631,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA29" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB29" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="30">
       <c r="A30" s="4">
@@ -3494,6 +3730,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA30" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB30" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="31">
       <c r="A31" s="4">
@@ -3585,6 +3829,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA31" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB31" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="32">
       <c r="A32" s="4">
@@ -3676,6 +3928,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA32" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB32" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="33">
       <c r="A33" s="4">
@@ -3767,6 +4027,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA33" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB33" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="34">
       <c r="A34" s="4">
@@ -3858,6 +4126,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA34" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB34" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="35">
       <c r="A35" s="4">
@@ -3949,6 +4225,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA35" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB35" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="36">
       <c r="A36" s="4">
@@ -4043,6 +4327,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA36" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB36" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="37">
       <c r="A37" s="4">
@@ -4137,6 +4429,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA37" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB37" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="38">
       <c r="A38" s="4">
@@ -4231,6 +4531,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA38" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB38" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="39">
       <c r="A39" s="4">
@@ -4325,6 +4633,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA39" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB39" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="40">
       <c r="A40" s="4">
@@ -4419,6 +4735,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA40" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB40" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="41">
       <c r="A41" s="4">
@@ -4513,6 +4837,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA41" s="12">
+        <v>2</v>
+      </c>
+      <c r="AB41" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="42">
       <c r="A42" s="4">
@@ -4607,6 +4939,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA42" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB42" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="43">
       <c r="A43" s="4">
@@ -4701,6 +5041,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA43" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB43" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="44">
       <c r="A44" s="4">
@@ -4795,6 +5143,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA44" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB44" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="45">
       <c r="A45" s="4">
@@ -4889,6 +5245,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA45" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB45" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="46">
       <c r="A46" s="4">
@@ -4983,6 +5347,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA46" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB46" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="47">
       <c r="A47" s="4">
@@ -5077,6 +5449,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA47" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB47" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="48">
       <c r="A48" s="4">
@@ -5171,6 +5551,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA48" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB48" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="49">
       <c r="A49" s="4">
@@ -5265,6 +5653,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA49" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB49" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="50">
       <c r="A50" s="4">
@@ -5359,6 +5755,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA50" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB50" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="51">
       <c r="A51" s="4">
@@ -5453,6 +5857,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA51" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB51" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="52">
       <c r="A52" s="4">
@@ -5547,6 +5959,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA52" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB52" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="53">
       <c r="A53" s="4">
@@ -5641,6 +6061,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA53" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB53" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="54">
       <c r="A54" s="4">
@@ -5735,6 +6163,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA54" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB54" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="55">
       <c r="A55" s="4">
@@ -5829,6 +6265,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA55" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB55" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="56">
       <c r="A56" s="4">
@@ -5920,6 +6364,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA56" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB56" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="57">
       <c r="A57" s="4">
@@ -6011,6 +6463,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA57" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB57" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="58">
       <c r="A58" s="4">
@@ -6102,6 +6562,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA58" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB58" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="59">
       <c r="A59" s="4">
@@ -6196,6 +6664,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA59" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB59" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="60">
       <c r="A60" s="4">
@@ -6290,6 +6766,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA60" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB60" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="61">
       <c r="A61" s="4">
@@ -6384,6 +6868,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA61" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB61" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="62">
       <c r="A62" s="4">
@@ -6475,6 +6967,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA62" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB62" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="63">
       <c r="A63" s="4">
@@ -6569,6 +7069,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA63" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB63" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="64">
       <c r="A64" s="4">
@@ -6663,6 +7171,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA64" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB64" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="65">
       <c r="A65" s="4">
@@ -6757,6 +7273,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA65" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB65" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="66">
       <c r="A66" s="4">
@@ -6851,6 +7375,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA66" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB66" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="67">
       <c r="A67" s="4">
@@ -6945,6 +7477,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA67" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB67" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="68">
       <c r="A68" s="4">
@@ -7039,6 +7579,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA68" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB68" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="69">
       <c r="A69" s="4">
@@ -7133,6 +7681,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA69" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB69" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="70">
       <c r="A70" s="4">
@@ -7227,6 +7783,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA70" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB70" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="71">
       <c r="A71" s="4">
@@ -7321,6 +7885,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA71" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB71" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="72">
       <c r="A72" s="4">
@@ -7415,6 +7987,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA72" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB72" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="73">
       <c r="A73" s="4">
@@ -7509,6 +8089,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA73" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB73" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="74">
       <c r="A74" s="4">
@@ -7603,6 +8191,14 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AA74" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB74" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="75">
       <c r="A75" s="4">
@@ -7697,6 +8293,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AB75" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="76">
       <c r="A76" s="4">
@@ -7791,6 +8392,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="AB76" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row outlineLevel="0" r="77">
       <c r="A77" s="4">
@@ -7883,6 +8489,11 @@
       <c r="Z77" s="5" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="AB77" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>

</xml_diff>